<commit_message>
Generalize multi-seat filter across all sources, not just OpenElections
The OE-only filter let multi-seat races leak through from every other
source: 'School Director Mt Lebanon' (WPRDC), 'Delegates To The National
Convention' (OE plural form the singular-only regex missed), 'SCH DIR
Directors At Large' (Lycoming abbreviation), 'Bradford City Study
Commission' (Vote For 7-9). Renamed _is_likely_multiseat_oe_race to
_is_likely_multiseat_race, broadened the regex to cover plurals
(directors?, delegates?, commissioners?), the SCH DIR abbreviation, and
study commissions, and lifted it to filter_likely_multiseat_races so it
runs as a final pipeline filter on every source. Drops Top_RCV_Races
from 303 to 242 non-majority races with the canonical Allentown 2021
DEM Mayor (Tuerk) still surfaced.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Philadelphia_Primary_Mayor_DistrictCouncil.xlsx
+++ b/Philadelphia_Primary_Mayor_DistrictCouncil.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="17">
   <si>
     <t>Candidate</t>
   </si>
@@ -32,27 +32,6 @@
     <t>Percent</t>
   </si>
   <si>
-    <t>CURTIS J JONES JR</t>
-  </si>
-  <si>
-    <t>CAROL ANN CAMPBELL</t>
-  </si>
-  <si>
-    <t>MATTHEW N MCCLURE</t>
-  </si>
-  <si>
-    <t>DONNA   REED MILLER</t>
-  </si>
-  <si>
-    <t>CINDY M BASS</t>
-  </si>
-  <si>
-    <t>IRV   ACKELSBERG</t>
-  </si>
-  <si>
-    <t>GREG   PAULMIER</t>
-  </si>
-  <si>
     <t>MICHAEL   NUTTER</t>
   </si>
   <si>
@@ -68,61 +47,7 @@
     <t>DWIGHT   EVANS</t>
   </si>
   <si>
-    <t>DISTRICT COUNCIL 4TH DISTRICT - D</t>
-  </si>
-  <si>
-    <t>DISTRICT COUNCIL 8TH DISTRICT - D</t>
-  </si>
-  <si>
     <t>MAYOR - D</t>
-  </si>
-  <si>
-    <t>MARK F SQUILLA</t>
-  </si>
-  <si>
-    <t>JOSEPH M GRACE</t>
-  </si>
-  <si>
-    <t>JEFF   HORNSTEIN</t>
-  </si>
-  <si>
-    <t>VERN   ANASTASIO</t>
-  </si>
-  <si>
-    <t>KENYATTA   JOHNSON</t>
-  </si>
-  <si>
-    <t>BARBARA A CAPOZZI</t>
-  </si>
-  <si>
-    <t>TRACEY   GORDON</t>
-  </si>
-  <si>
-    <t>DAMON K ROBERTS</t>
-  </si>
-  <si>
-    <t>VERNA   TYNER</t>
-  </si>
-  <si>
-    <t>HOWARD   TREATMAN</t>
-  </si>
-  <si>
-    <t>ROBIN M TASCO</t>
-  </si>
-  <si>
-    <t>ANDREW   LOFTON</t>
-  </si>
-  <si>
-    <t>WILLIAM A DURHAM JR</t>
-  </si>
-  <si>
-    <t>DISTRICT COUNCIL 1ST DIST - DEM</t>
-  </si>
-  <si>
-    <t>DISTRICT COUNCIL 2ND DIST - DEM</t>
-  </si>
-  <si>
-    <t>DISTRICT COUNCIL 8TH DIST - DEM</t>
   </si>
   <si>
     <t>CHERELLE L PARKER</t>
@@ -501,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -523,13 +448,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C2">
-        <v>9144</v>
+        <v>106805</v>
       </c>
       <c r="D2">
-        <v>34.87015215650383</v>
+        <v>36.64230822011802</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -537,13 +462,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C3">
-        <v>8674</v>
+        <v>71731</v>
       </c>
       <c r="D3">
-        <v>33.07783243717347</v>
+        <v>24.60923562508577</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -551,138 +476,40 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C4">
-        <v>8304</v>
+        <v>44474</v>
       </c>
       <c r="D4">
-        <v>31.66685733897723</v>
+        <v>15.2579936873885</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5">
+        <v>44301</v>
+      </c>
+      <c r="D5">
+        <v>15.19864141622067</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C6">
-        <v>9735</v>
+        <v>22782</v>
       </c>
       <c r="D6">
-        <v>31.57945956466734</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7">
-        <v>8170</v>
-      </c>
-      <c r="D7">
-        <v>26.50274110357803</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8">
-        <v>7783</v>
-      </c>
-      <c r="D8">
-        <v>25.24734810393486</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9">
-        <v>5106</v>
-      </c>
-      <c r="D9">
-        <v>16.56340221234632</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11">
-        <v>106805</v>
-      </c>
-      <c r="D11">
-        <v>36.64230822011802</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12">
-        <v>71731</v>
-      </c>
-      <c r="D12">
-        <v>24.60923562508577</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13">
-        <v>44474</v>
-      </c>
-      <c r="D13">
-        <v>15.2579936873885</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14">
-        <v>44301</v>
-      </c>
-      <c r="D14">
-        <v>15.19864141622067</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15">
-        <v>22782</v>
-      </c>
-      <c r="D15">
         <v>7.815973651708521</v>
       </c>
     </row>
@@ -693,7 +520,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -708,216 +535,6 @@
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2">
-        <v>7234</v>
-      </c>
-      <c r="D2">
-        <v>41.04164302734596</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3">
-        <v>4074</v>
-      </c>
-      <c r="D3">
-        <v>23.11358220810167</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4">
-        <v>3511</v>
-      </c>
-      <c r="D4">
-        <v>19.91943719505277</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5">
-        <v>2807</v>
-      </c>
-      <c r="D5">
-        <v>15.9253375694996</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7">
-        <v>7486</v>
-      </c>
-      <c r="D7">
-        <v>44.49595815501664</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8">
-        <v>7446</v>
-      </c>
-      <c r="D8">
-        <v>44.25820256776034</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9">
-        <v>1566</v>
-      </c>
-      <c r="D9">
-        <v>9.308131241084165</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10">
-        <v>326</v>
-      </c>
-      <c r="D10">
-        <v>1.937708036138849</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12">
-        <v>8883</v>
-      </c>
-      <c r="D12">
-        <v>39.37674542311272</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13">
-        <v>4796</v>
-      </c>
-      <c r="D13">
-        <v>21.2598076155858</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14">
-        <v>4185</v>
-      </c>
-      <c r="D14">
-        <v>18.55135422669445</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15">
-        <v>2950</v>
-      </c>
-      <c r="D15">
-        <v>13.07682078106299</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16">
-        <v>735</v>
-      </c>
-      <c r="D16">
-        <v>3.258123143756372</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17">
-        <v>637</v>
-      </c>
-      <c r="D17">
-        <v>2.823706724588856</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18">
-        <v>373</v>
-      </c>
-      <c r="D18">
-        <v>1.653442085198812</v>
       </c>
     </row>
   </sheetData>
@@ -994,10 +611,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>162160</v>
@@ -1008,10 +625,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C3">
         <v>113162</v>
@@ -1022,10 +639,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C4">
         <v>109410</v>
@@ -1036,10 +653,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C5">
         <v>56102</v>
@@ -1050,10 +667,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>43736</v>
@@ -1064,10 +681,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>6642</v>

</xml_diff>